<commit_message>
auto: snapshot 2026-09-14 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -58,6 +58,7 @@
     <sheet name="2026-09-11" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="2026-09-12" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="2026-09-13" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="2026-09-14" sheetId="52" state="visible" r:id="rId52"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -42219,6 +42220,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-14 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>25297</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>379</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>6672</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>178</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2975</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>23216</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+5712</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ZÎ£ WHITÎ£BÎ£ARD</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>476</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+476</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>AangEX2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>5520</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>8409</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>SeeYuSoon</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>2184</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6474</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1023</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>35558</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1008</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>21360</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>32941</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | $ignature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>5074</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>1260</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>16002</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>4528</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>7162</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>52941</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+7896</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>43140</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+8217</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>10283</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1084</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-14 05:30:26
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -42250,11 +42250,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-14 13:00:10</t>
+          <t>Timestamp: 2026-09-14 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>25297</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3">
@@ -43001,11 +43001,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>52941</v>
+        <v>53025</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+7896</t>
+          <t>+7980</t>
         </is>
       </c>
     </row>
@@ -43046,11 +43046,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>43140</v>
+        <v>43224</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+8217</t>
+          <t>+8301</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-14 05:45:39
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -42250,11 +42250,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-14 13:30:25</t>
+          <t>Timestamp: 2026-09-14 13:45:38</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>168</v>
+        <v>336</v>
       </c>
     </row>
     <row r="3">
@@ -43001,11 +43001,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>53025</v>
+        <v>53109</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+7980</t>
+          <t>+8064</t>
         </is>
       </c>
     </row>
@@ -43046,11 +43046,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>43224</v>
+        <v>43308</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+8301</t>
+          <t>+8385</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-15 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -59,6 +59,7 @@
     <sheet name="2026-09-12" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="2026-09-13" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="2026-09-14" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="2026-09-15" sheetId="53" state="visible" r:id="rId53"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43108,6 +43109,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-15 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>13446</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>379</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>6672</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>206</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2975</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>24980</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+1764</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ZÎ£ WHITÎ£BÎ£ARD</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>476</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>AangEX2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>5520</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+1024</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>8409</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>SeeYuSoon</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>2198</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+14</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6894</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1443</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>35978</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>21360</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>33361</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | $ignature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+14</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>318</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+318</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>5494</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>1680</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>16002</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>4528</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>321</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+321</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>7162</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>56973</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+3864</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>46131</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2823</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>10283</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1504</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-15 05:30:28
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -43139,11 +43139,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-15 13:00:10</t>
+          <t>Timestamp: 2026-09-15 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>13446</v>
+        <v>13698</v>
       </c>
     </row>
     <row r="3">
@@ -43260,11 +43260,11 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>24980</v>
+        <v>25064</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>+1764</t>
+          <t>+1848</t>
         </is>
       </c>
     </row>
@@ -43890,11 +43890,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>56973</v>
+        <v>57057</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+3864</t>
+          <t>+3948</t>
         </is>
       </c>
     </row>
@@ -43935,11 +43935,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>46131</v>
+        <v>46215</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2823</t>
+          <t>+2907</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-16 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -60,6 +60,7 @@
     <sheet name="2026-09-13" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="2026-09-14" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="2026-09-15" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="2026-09-16" sheetId="54" state="visible" r:id="rId54"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43997,6 +43998,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-16 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>10916</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>f0rgotten</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>805</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+14</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>4984</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>26828</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1764</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>ZÎ£ WHITÎ£BÎ£ARD</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>476</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>AangEX2</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>7122</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+1602</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>8409</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>SeeYouSoon</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>2254</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>416</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+366</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>6894</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1443</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>35978</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>21360</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>33361</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | $ignature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>318</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>5494</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2048</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+368</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+14</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>16002</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>4528</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>321</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>7162</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>60719</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3662</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>RS | Oboy Max</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>3030</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>48443</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2228</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>10283</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1504</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-16 05:30:28
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -44028,11 +44028,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-16 13:00:10</t>
+          <t>Timestamp: 2026-09-16 13:30:26</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>10916</v>
+        <v>11174</v>
       </c>
     </row>
     <row r="3">
@@ -44119,11 +44119,11 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>4984</v>
+        <v>5068</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>+2009</t>
+          <t>+2093</t>
         </is>
       </c>
     </row>
@@ -44209,11 +44209,11 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>7122</v>
+        <v>7206</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>+1602</t>
+          <t>+1686</t>
         </is>
       </c>
     </row>
@@ -44764,11 +44764,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>60719</v>
+        <v>60725</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3662</t>
+          <t>+3668</t>
         </is>
       </c>
     </row>
@@ -44809,7 +44809,7 @@
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>3030</v>
+        <v>3114</v>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-17 05:00:14
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -61,6 +61,7 @@
     <sheet name="2026-09-14" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="2026-09-15" sheetId="53" state="visible" r:id="rId53"/>
     <sheet name="2026-09-16" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="2026-09-17" sheetId="55" state="visible" r:id="rId55"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -44886,6 +44887,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-17 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>12683</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>f0rgotten</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>805</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6637</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+1569</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>28430</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1602</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>ZÎ£ WHITÎ£BÎ£ARD</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>476</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>AangEX2</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>8814</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+1608</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>8409</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>SeeYouSoon</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>2254</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>836</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>C.L.A.Z</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>8467</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+1573</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1920</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+477</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>36398</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>21360</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>33781</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | $ignature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SESSHOMARU</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>318</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>6723</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+1229</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2048</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>16002</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>4528</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>321</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>7162</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>64478</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3753</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>RS | Oboy Max</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>6750</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+3636</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>51497</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3054</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>10283</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1504</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-17 05:30:28
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -44917,11 +44917,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-17 13:00:12</t>
+          <t>Timestamp: 2026-09-17 13:30:26</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>12683</v>
+        <v>191</v>
       </c>
     </row>
     <row r="3">
@@ -45278,11 +45278,11 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>8467</v>
+        <v>8499</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>+1573</t>
+          <t>+1605</t>
         </is>
       </c>
     </row>
@@ -45503,11 +45503,11 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>6723</v>
+        <v>6729</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>+1229</t>
+          <t>+1235</t>
         </is>
       </c>
     </row>
@@ -45653,11 +45653,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>64478</v>
+        <v>64562</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3753</t>
+          <t>+3837</t>
         </is>
       </c>
     </row>
@@ -45698,11 +45698,11 @@
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>6750</v>
+        <v>6823</v>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>+3636</t>
+          <t>+3709</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-18 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -62,6 +62,7 @@
     <sheet name="2026-09-15" sheetId="53" state="visible" r:id="rId53"/>
     <sheet name="2026-09-16" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="2026-09-17" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="2026-09-18" sheetId="56" state="visible" r:id="rId56"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45775,6 +45776,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-18 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>16006</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>f0rgotten</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>805</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>865</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+645</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>9454</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+2817</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>30032</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1602</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>ZÎ£ WHITÎ£BÎ£ARD</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>476</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>AangEX2</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>8814</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>851</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+851</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>8409</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>SeeYouSoon</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>2254</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>836</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>C.L.A.Z</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>8885</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+386</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1920</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>36818</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>21360</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>675</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>34201</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | $ignature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SESSHOMARU</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>318</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>6940</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+211</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2048</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>16002</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>4528</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>321</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>7164</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>68250</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3688</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>RS | Oboy Max</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>8157</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+1334</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>54261</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2764</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>10283</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1504</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-18 05:30:24
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -45806,11 +45806,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-18 13:00:11</t>
+          <t>Timestamp: 2026-09-18 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>16006</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -46542,11 +46542,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>68250</v>
+        <v>68334</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3688</t>
+          <t>+3772</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-19 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -63,6 +63,7 @@
     <sheet name="2026-09-16" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="2026-09-17" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="2026-09-18" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="2026-09-19" sheetId="57" state="visible" r:id="rId57"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46664,6 +46665,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-19 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>f0rgotten</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>805</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>866</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>9454</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>31544</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1512</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>ZÎ£ WHITÎ£BÎ£ARD</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>476</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>AangEX2</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>8814</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>851</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>8409</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>SeeYouSoon</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>2268</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+14</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>836</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>C.L.A.Z</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>8885</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>2340</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Suhaib</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>37238</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>21360</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>675</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>34621</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | $ignature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SESSHOMARU</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>318</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>6940</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2048</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>16002</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>4528</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Mode pilot</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>321</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>7164</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>72269</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3935</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>RS | Oboy Max</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>9630</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+1473</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>57637</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3376</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>10283</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>2008</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+504</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-19 05:30:28
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -46695,7 +46695,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-19 13:00:11</t>
+          <t>Timestamp: 2026-09-19 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
@@ -46996,11 +46996,11 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>2268</v>
+        <v>2352</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>+14</t>
+          <t>+98</t>
         </is>
       </c>
     </row>
@@ -47082,7 +47082,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Suhaib</t>
+          <t>Ryujin</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
@@ -47431,11 +47431,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>72269</v>
+        <v>72383</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3935</t>
+          <t>+4049</t>
         </is>
       </c>
     </row>
@@ -47476,11 +47476,11 @@
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>9630</v>
+        <v>9661</v>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>+1473</t>
+          <t>+1504</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-20 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -64,6 +64,7 @@
     <sheet name="2026-09-17" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="2026-09-18" sheetId="56" state="visible" r:id="rId56"/>
     <sheet name="2026-09-19" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="2026-09-20" sheetId="58" state="visible" r:id="rId58"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47553,6 +47554,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-20 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>21241</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+21241</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>f0rgotten</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20875</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+20070</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>17641</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+17641</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>23444</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+22578</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>33144</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+23690</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>54603</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+23059</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>21731</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+21731</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>20480</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+19660</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>ZÎ£ WHITÎ£BÎ£ARD</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>20302</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+19826</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>27235</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+27235</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>AangEX2</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>29760</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+20946</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>22165</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+22165</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>21043</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+20192</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>21770</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+21770</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>22106</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+21082</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>20151</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>28768</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+20359</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>19887</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+19887</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>SeeYouSoon</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>25992</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+23640</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>21235</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+20399</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>10610</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+10610</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>C.L.A.Z</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>22101</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+22101</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>29102</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+20217</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>24795</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+22455</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>20393</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+20393</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>118297</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+118297</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>63791</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+26553</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>42409</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+21049</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>112630</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+112630</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Me®u</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>28272</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>57750</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+23129</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | $ignature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>10178</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+10178</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>9199</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+9199</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshõmaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>21998</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>19193</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+19144</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>21763</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+21763</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>22323</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+22005</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>29020</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+22080</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>18708</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+18708</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>22814</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+20766</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>19852</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+19852</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>21772</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+21772</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>21521</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+21507</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>39891</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+23889</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>26527</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+21999</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>20614</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>27357</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+20193</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>98821</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+26438</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>22153</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+21481</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>21244</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+21216</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>RS | Oboy Max</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>35255</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+25594</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>83918</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+26281</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>20947</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+20947</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>30054</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+19771</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>22085</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+20077</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-20 05:30:25
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -47584,7 +47584,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-20 13:00:11</t>
+          <t>Timestamp: 2026-09-20 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
@@ -47881,7 +47881,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>SeeYouSoon</t>
+          <t>SNC | Asuna</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
@@ -47889,7 +47889,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>+23640</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>